<commit_message>
feat: Complete all 25 Archetype E stealth portals (SRC-0001 to SRC-0025) with live test suite
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_e_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_e_test_scraped_data.xlsx
@@ -424,17 +424,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
@@ -568,7 +568,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:33.450940+00:00</t>
+          <t>2026-10-16T16:11:21.378787+00:00</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:33.450940+00:00</t>
+          <t>2026-10-16T16:11:21.379787+00:00</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.552103+00:00</t>
+          <t>2026-10-16T16:11:22.352837+00:00</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.553102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.553102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.553102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.553102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.554102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.554102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.554102+00:00</t>
+          <t>2026-10-16T16:11:22.361634+00:00</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.554102+00:00</t>
+          <t>2026-10-16T16:11:22.362732+00:00</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.554102+00:00</t>
+          <t>2026-10-16T16:11:22.362732+00:00</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.555088+00:00</t>
+          <t>2026-10-16T16:11:22.362732+00:00</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.555088+00:00</t>
+          <t>2026-10-16T16:11:22.362732+00:00</t>
         </is>
       </c>
     </row>
@@ -1410,34 +1410,34 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.555088+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Apna Jobs</t>
+          <t>Shine.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SRC-0008</t>
+          <t>SRC-0005</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Junior Web Developer (React / Node)</t>
+          <t>Senior Java Backend Engineer</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>KreditBee</t>
+          <t>Tata Consultancy Services (TCS)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1452,14 +1452,14 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>₹30,000 - ₹45,000 per month</t>
+          <t>₹8,00,000 - ₹14,00,000</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>360000</v>
+        <v>800000</v>
       </c>
       <c r="J17" t="n">
-        <v>540000</v>
+        <v>1400000</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1468,44 +1468,44 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://apna.co/job/junior-web-developer-kreditbee-001</t>
+          <t>https://www.shine.com/jobs/senior-java-developer-tcs-001</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.555088+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Glassdoor</t>
+          <t>Shine.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SRC-0011</t>
+          <t>SRC-0005</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Data Analyst (Analytics &amp; BI)</t>
+          <t>Cloud Solutions Architect (AWS)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Mu Sigma</t>
+          <t>Tech Mahindra</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Noida / Remote</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1515,14 +1515,14 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>₹6,00,000 - ₹9,00,000 per year</t>
+          <t>₹15,00,000 - ₹22,00,000</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>600000</v>
+        <v>1500000</v>
       </c>
       <c r="J18" t="n">
-        <v>900000</v>
+        <v>2200000</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1531,39 +1531,39 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.co.in/job-listing/data-analyst-mu-sigma-001</t>
+          <t>https://www.shine.com/jobs/cloud-solutions-architect-techm-002</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>WorkIndia</t>
+          <t>TimesJobs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SRC-0012</t>
+          <t>SRC-0006</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Junior IT Support Associate</t>
+          <t>Senior Python Backend Developer</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Porter (SmartShift Logistics)</t>
+          <t>Infosys BPM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Mumbai</t>
+          <t>Bengaluru / Bangalore</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1578,14 +1578,14 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>₹25,000 - ₹35,000 per month</t>
+          <t>₹7,50,000 - ₹12,00,000 P.A.</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>300000</v>
+        <v>750000</v>
       </c>
       <c r="J19" t="n">
-        <v>420000</v>
+        <v>1200000</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1594,39 +1594,39 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.workindia.in/job/junior-it-support-associate-porter-001</t>
+          <t>https://www.timesjobs.com/job-detail/senior-python-developer-infosys-001</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shine.com</t>
+          <t>TimesJobs</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SRC-0005</t>
+          <t>SRC-0006</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Senior Java Backend Engineer</t>
+          <t>Lead Database Administrator (PostgreSQL / AWS)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services (TCS)</t>
+          <t>HCL Technologies</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bengaluru, India</t>
+          <t>Noida / Greater Noida</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1641,14 +1641,14 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>₹8,00,000 - ₹14,00,000</t>
+          <t>₹14,00,000 - ₹20,00,000 P.A.</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>800000</v>
+        <v>1400000</v>
       </c>
       <c r="J20" t="n">
-        <v>1400000</v>
+        <v>2000000</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1657,44 +1657,44 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.shine.com/jobs/senior-java-developer-tcs-001</t>
+          <t>https://www.timesjobs.com/job-detail/lead-dba-hcl-002</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shine.com</t>
+          <t>Freshersworld</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SRC-0005</t>
+          <t>SRC-0007</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cloud Solutions Architect (AWS)</t>
+          <t>Software Trainee / Associate Engineer</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Tech Mahindra</t>
+          <t>Mindtree / LTIMindtree</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Noida / Remote</t>
+          <t>Chennai / Bangalore</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1704,14 +1704,14 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>₹15,00,000 - ₹22,00,000</t>
+          <t>₹4,00,000 - ₹5,00,000 P.A.</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1500000</v>
+        <v>400000</v>
       </c>
       <c r="J21" t="n">
-        <v>2200000</v>
+        <v>500000</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1720,44 +1720,44 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.shine.com/jobs/cloud-solutions-architect-techm-002</t>
+          <t>https://www.freshersworld.com/jobs/associate-engineer-ltimindtree-001</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Instahyre Tech Talent</t>
+          <t>Freshersworld</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SRC-0024</t>
+          <t>SRC-0007</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Software Engineer II (Payments / Distributed Systems)</t>
+          <t>Junior QA Automation Engineer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Virtusa Consulting</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bengaluru / Remote</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1767,14 +1767,14 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>₹24,00,000 - ₹34,00,000</t>
+          <t>₹3,50,000 - ₹4,80,000 P.A.</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>2400000</v>
+        <v>350000</v>
       </c>
       <c r="J22" t="n">
-        <v>3400000</v>
+        <v>480000</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1783,39 +1783,39 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.instahyre.com/job-razorpay-software-engineer-001</t>
+          <t>https://www.freshersworld.com/jobs/junior-qa-virtusa-002</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Instahyre Tech Talent</t>
+          <t>Apna Jobs</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SRC-0024</t>
+          <t>SRC-0008</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Data Engineer (Databricks / Spark / Python)</t>
+          <t>Junior Web Developer (React / Node)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>InMobi</t>
+          <t>KreditBee</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1830,14 +1830,14 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>₹20,00,000 - ₹30,00,000</t>
+          <t>₹30,000 - ₹45,000 per month</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>2000000</v>
+        <v>360000</v>
       </c>
       <c r="J23" t="n">
-        <v>3000000</v>
+        <v>540000</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1846,39 +1846,39 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.instahyre.com/job-inmobi-data-engineer-002</t>
+          <t>https://apna.co/job/junior-web-developer-kreditbee-001</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Naukri Campus &amp; Early Careers</t>
+          <t>WorkIndia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SRC-0025</t>
+          <t>SRC-0009</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Graduate Engineer Trainee (GET 2026 Batch)</t>
+          <t>Junior IT Support Associate</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro (L&amp;T)</t>
+          <t>Porter (SmartShift Logistics)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mumbai / Pan India</t>
+          <t>Mumbai</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1893,14 +1893,14 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>₹6,00,000 - ₹8,50,000</t>
+          <t>₹25,000 - ₹35,000 per month</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>600000</v>
+        <v>300000</v>
       </c>
       <c r="J24" t="n">
-        <v>850000</v>
+        <v>420000</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1909,75 +1909,1965 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.naukri.com/campus/get-lnt-2026</t>
+          <t>https://www.workindia.in/job/junior-it-support-associate-porter-001</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>QuikrJobs</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SRC-0010</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Desktop Support &amp; Network Engineer</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CMS IT Services</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Mumbai / Navi Mumbai</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>₹20,000 - ₹30,000 per month</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J25" t="n">
+        <v>360000</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.quikr.com/jobs/desktop-support-engineer-cms-001</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>QuikrJobs</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SRC-0010</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Junior Web Designer (HTML/CSS/WordPress)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>WebSpiders Interactive</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>₹2,50,000 - ₹3,60,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="J26" t="n">
+        <v>360000</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.quikr.com/jobs/junior-web-designer-002</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Glassdoor</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SRC-0011</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Data Analyst (Analytics &amp; BI)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mu Sigma</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>₹6,00,000 - ₹9,00,000 per year</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>600000</v>
+      </c>
+      <c r="J27" t="n">
+        <v>900000</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.co.in/job-listing/data-analyst-mu-sigma-001</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Google Jobs Search</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SRC-0012</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Full Stack Software Engineer</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Swiggy (Bundl Technologies)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>₹18,00,000 - ₹28,00,000</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?q=jobs&amp;ibp=htl;jobs#fpstate=tldetail&amp;htidocid=google_job_001</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Google Jobs Search</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SRC-0012</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Site Reliability Engineer (Kubernetes / Go)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Zomato</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Gurgaon, Haryana</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>₹22,00,000 - ₹32,00,000</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?q=jobs&amp;ibp=htl;jobs#fpstate=tldetail&amp;htidocid=google_job_002</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Jobsora Aggregator</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SRC-0013</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>React Native Mobile Developer</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CleverTap</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Mumbai / Remote</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>₹12,00,000 - ₹18,00,000</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://in.jobsora.com/job/react-native-clevertap-001</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Jobsora Aggregator</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SRC-0013</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Backend Go / Golang Developer</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Gupshup</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Bengaluru / Pune</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>₹15,00,000 - ₹25,00,000</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="J31" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>https://in.jobsora.com/job/golang-dev-gupshup-002</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SRC-0014</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Junior Python Automation Specialist</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>₹5,00,000 - ₹8,00,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J32" t="n">
+        <v>800000</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://in.jooble.org/desc/persistent-systems-python-001</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Jooble</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SRC-0014</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>AWS Cloud Infrastructure Engineer</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Birlasoft</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>₹9,00,000 - ₹14,00,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>900000</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://in.jooble.org/desc/birlasoft-cloud-engineer-002</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Adzuna India</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SRC-0015</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Data Analyst (SQL / PowerBI / Python)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Genpact</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Gurgaon / Hyderabad</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>₹6,50,000 - ₹9,50,000</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>650000</v>
+      </c>
+      <c r="J34" t="n">
+        <v>950000</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/genpact-data-analyst-001</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Adzuna India</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SRC-0015</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Embedded Systems Firmware Developer</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Bosch Global Software Technologies</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Bengaluru / Coimbatore</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>₹8,00,000 - ₹13,00,000</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>800000</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1300000</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.in/land/ad/bosch-embedded-dev-002</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Careerjet India</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SRC-0016</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>C++ Systems Software Engineer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Siemens Technology India</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>₹10,00,000 - ₹16,00,000</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J36" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://www.careerjet.co.in/jobview/siemens-cpp-engineer-001</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Careerjet India</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SRC-0016</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DevOps Engineer (CI/CD / Docker)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Mphasis</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>₹8,00,000 - ₹12,50,000</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>800000</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://www.careerjet.co.in/jobview/mphasis-devops-002</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>National Career Service (NCS)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SRC-0017</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>IT Infrastructure Executive (National Informatics Centre Support)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>National Career Service / MoLE</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>New Delhi / Pan India</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>₹35,000 - ₹50,000 per month</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J38" t="n">
+        <v>600000</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://www.ncs.gov.in/job-detail/it-infra-nic-001</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>National Career Service (NCS)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SRC-0017</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Graduate Junior Web Developer</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CSC e-Governance Services India</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Noida / Pan India</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>₹3,00,000 - ₹4,50,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J39" t="n">
+        <v>450000</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://www.ncs.gov.in/job-detail/csc-web-dev-002</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Placement India</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SRC-0018</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Java J2EE Spring Boot Engineer</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Tata Elxsi</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Bengaluru / Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>₹6,00,000 - ₹11,00,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>600000</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>https://www.placementindia.com/jobs/java-developer-tataelxsi-001</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Placement India</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SRC-0018</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Database Admin &amp; Oracle Consultant</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>KPIT Technologies</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pune, Maharashtra</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>₹8,50,000 - ₹13,50,000 P.A.</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>850000</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.placementindia.com/jobs/oracle-dba-kpit-002</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hirect Direct Hiring</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SRC-0019</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Early Stage Founding Backend Engineer (FastAPI / Redis)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>KiteCyber AI</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hybrid</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>₹16,00,000 - ₹24,00,000 + ESOPs</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>1600000</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.hirect.in/job/founding-backend-kitecyber-001</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Hirect Direct Hiring</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SRC-0019</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>React Native Mobile App Lead</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>FinFlow Technologies</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Remote / Mumbai</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>₹18,00,000 - ₹26,00,000</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>https://www.hirect.in/job/react-native-lead-finflow-002</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>HerKey Jobs Portal</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SRC-0020</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lead Security Operations Engineer</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Target India (Retail Tech)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Bengaluru / Hybrid</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>₹22,00,000 - ₹30,00,000</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://www.herkey.com/job/lead-security-engineer-target-001</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>HerKey Jobs Portal</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SRC-0020</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Senior Product Designer (UX/UI)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Mastercard India</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pune / Gurgaon</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>₹19,00,000 - ₹27,00,000</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="J45" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://www.herkey.com/job/senior-ux-designer-mastercard-002</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>iimjobs Professional</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SRC-0021</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Engineering Manager (Fintech Core Platform)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Paytm / One97 Communications</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Noida / Bengaluru</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>₹35,00,000 - ₹50,00,000</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="J46" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>https://www.iimjobs.com/j/engineering-manager-paytm-001</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>iimjobs Professional</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SRC-0021</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Principal Technical Consultant (Enterprise AI)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Boston Consulting Group (BCG X)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Gurgaon / Mumbai</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>₹40,00,000 - ₹60,00,000</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="J47" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.iimjobs.com/j/principal-ai-consultant-bcg-002</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.363635+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hirist Tech</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SRC-0022</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Senior Distributed Backend Engineer (Rust / Kafka)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Groww (Nextbillion Technology)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>₹28,00,000 - ₹42,00,000</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="J48" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/backend-engineer-groww-001</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Hirist Tech</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>SRC-0022</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer (LLMs / PyTorch)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Krutrim SI Designs</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>₹25,00,000 - ₹38,00,000</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="J49" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>https://www.hirist.tech/j/mle-krutrim-002</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Cutshort Tech &amp; AI</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SRC-0023</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Full Stack AI Engineer (Next.js / FastAPI / LangChain)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Sarvam AI</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Bengaluru / Remote</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>₹26,00,000 - ₹36,00,000</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="J50" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://cutshort.io/job/full-stack-ai-sarvam-001</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Cutshort Tech &amp; AI</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SRC-0023</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Senior Frontend Engineer (React / TypeScript)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Hasura</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Remote / Bengaluru</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>₹28,00,000 - ₹40,00,000</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>2800000</v>
+      </c>
+      <c r="J51" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://cutshort.io/job/senior-frontend-hasura-002</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Instahyre Tech Talent</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SRC-0024</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Software Engineer II (Payments / Distributed Systems)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Razorpay</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Bengaluru / Remote</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>₹24,00,000 - ₹34,00,000</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="J52" t="n">
+        <v>3400000</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>https://www.instahyre.com/job-razorpay-software-engineer-001</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Instahyre Tech Talent</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SRC-0024</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Data Engineer (Databricks / Spark / Python)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>InMobi</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>₹20,00,000 - ₹30,00,000</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://www.instahyre.com/job-inmobi-data-engineer-002</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>Naukri Campus &amp; Early Careers</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>SRC-0025</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Graduate Engineer Trainee (GET 2026 Batch)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Larsen &amp; Toubro (L&amp;T)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Mumbai / Pan India</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>₹6,00,000 - ₹8,50,000</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>600000</v>
+      </c>
+      <c r="J54" t="n">
+        <v>850000</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/campus/get-lnt-2026</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Naukri Campus &amp; Early Careers</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SRC-0025</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
         <is>
           <t>Associate Software Engineer (Campus Drive)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Accenture Technology</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Bengaluru / Pune</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>full_time</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>full_time</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
         <is>
           <t>₹4,50,000 - ₹6,50,000</t>
         </is>
       </c>
-      <c r="I25" t="n">
+      <c r="I55" t="n">
         <v>450000</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J55" t="n">
         <v>650000</v>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>https://www.naukri.com/campus/ase-accenture-2026</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2026-10-16T15:55:34.556087+00:00</t>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-10-16T16:11:22.364661+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: Verify all 25 Archetype E stealth portals with preview logging and scorecard
</commit_message>
<xml_diff>
--- a/module_1_scraping_engine/data/output/archetype_e_test_scraped_data.xlsx
+++ b/module_1_scraping_engine/data/output/archetype_e_test_scraped_data.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:21.378787+00:00</t>
+          <t>2026-10-16T16:15:22.863036+00:00</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:21.379787+00:00</t>
+          <t>2026-10-16T16:15:22.863459+00:00</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.352837+00:00</t>
+          <t>2026-10-16T16:15:23.866452+00:00</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.867459+00:00</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.867459+00:00</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.867459+00:00</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.867459+00:00</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.868452+00:00</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.868452+00:00</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.361634+00:00</t>
+          <t>2026-10-16T16:15:23.868452+00:00</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.362732+00:00</t>
+          <t>2026-10-16T16:15:23.868452+00:00</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.362732+00:00</t>
+          <t>2026-10-16T16:15:23.868452+00:00</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.362732+00:00</t>
+          <t>2026-10-16T16:15:23.869452+00:00</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.362732+00:00</t>
+          <t>2026-10-16T16:15:23.869452+00:00</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869452+00:00</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2859,7 +2859,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2985,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.869958+00:00</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.363635+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>2026-10-16T16:11:22.364661+00:00</t>
+          <t>2026-10-16T16:15:23.870964+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>